<commit_message>
Corrigido bug no torneio de Nimbasa
</commit_message>
<xml_diff>
--- a/Docs/Encounter locations.xlsx
+++ b/Docs/Encounter locations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benit\Documents\GitHub\Pokemon Burning Scales\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benit\Documents\GitHub\Pokemon-Burning-Scales\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DB27E1C-B80D-49C2-A666-A6357C3F5CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8481988B-A5E2-4B9A-8F9C-EB7D3863ABF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="174">
   <si>
     <t>Pokemon</t>
   </si>
@@ -555,6 +555,9 @@
   </si>
   <si>
     <t>Dedenne</t>
+  </si>
+  <si>
+    <t>Relic Castle B7F</t>
   </si>
 </sst>
 </file>
@@ -1564,6 +1567,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1571,7 +1575,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2791,7 +2794,7 @@
         <v>64</v>
       </c>
       <c r="K10" t="s">
-        <v>65</v>
+        <v>173</v>
       </c>
       <c r="L10" t="s">
         <v>59</v>

</xml_diff>